<commit_message>
feat: generate and export daily global market data and monitor reports
</commit_message>
<xml_diff>
--- a/outputs/global_xlsx/global_market_20260324.xlsx
+++ b/outputs/global_xlsx/global_market_20260324.xlsx
@@ -468,16 +468,16 @@
         </is>
       </c>
       <c r="C2" t="n">
-        <v>6581</v>
+        <v>6556.37</v>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>1.15%</t>
+          <t>-0.37%</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>03/23</t>
+          <t>03/24</t>
         </is>
       </c>
     </row>
@@ -493,16 +493,16 @@
         </is>
       </c>
       <c r="C3" t="n">
-        <v>46208.47</v>
+        <v>46124.06</v>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>1.38%</t>
+          <t>-0.18%</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>03/23</t>
+          <t>03/24</t>
         </is>
       </c>
     </row>
@@ -518,16 +518,16 @@
         </is>
       </c>
       <c r="C4" t="n">
-        <v>21946.76</v>
+        <v>21761.89</v>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>1.38%</t>
+          <t>-0.84%</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>03/23</t>
+          <t>03/24</t>
         </is>
       </c>
     </row>
@@ -543,16 +543,16 @@
         </is>
       </c>
       <c r="C5" t="n">
-        <v>7773.13</v>
+        <v>7872.71</v>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>1.34%</t>
+          <t>1.28%</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>03/23</t>
+          <t>03/24</t>
         </is>
       </c>
     </row>
@@ -568,16 +568,16 @@
         </is>
       </c>
       <c r="C6" t="n">
-        <v>22653.86</v>
+        <v>22636.91</v>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>1.22%</t>
+          <t>-0.07%</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>03/23</t>
+          <t>03/24</t>
         </is>
       </c>
     </row>
@@ -593,16 +593,16 @@
         </is>
       </c>
       <c r="C7" t="n">
-        <v>7726.2</v>
+        <v>7743.92</v>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>0.79%</t>
+          <t>0.23%</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>03/23</t>
+          <t>03/24</t>
         </is>
       </c>
     </row>
@@ -618,16 +618,16 @@
         </is>
       </c>
       <c r="C8" t="n">
-        <v>9894.15</v>
+        <v>9965.16</v>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>-0.24%</t>
+          <t>0.72%</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>03/23</t>
+          <t>03/24</t>
         </is>
       </c>
     </row>
@@ -643,16 +643,16 @@
         </is>
       </c>
       <c r="C9" t="n">
-        <v>51886.42</v>
+        <v>54007.04</v>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>0.72%</t>
+          <t>4.84%</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>03/24</t>
+          <t>03/25</t>
         </is>
       </c>
     </row>
@@ -668,16 +668,16 @@
         </is>
       </c>
       <c r="C10" t="n">
-        <v>5428.97</v>
+        <v>5725.48</v>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>0.43%</t>
+          <t>5.91%</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>03/24</t>
+          <t>03/25</t>
         </is>
       </c>
     </row>
@@ -693,11 +693,11 @@
         </is>
       </c>
       <c r="C11" t="n">
-        <v>32680.41</v>
+        <v>32612.24</v>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>-0.13%</t>
+          <t>-0.34%</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
@@ -718,11 +718,11 @@
         </is>
       </c>
       <c r="C12" t="n">
-        <v>24605.93</v>
+        <v>25063.71</v>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>0.92%</t>
+          <t>2.79%</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
@@ -743,11 +743,11 @@
         </is>
       </c>
       <c r="C13" t="n">
-        <v>4415.45</v>
+        <v>4474.72</v>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>-0.06%</t>
+          <t>1.28%</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
@@ -768,16 +768,16 @@
         </is>
       </c>
       <c r="C14" t="n">
-        <v>8381.799999999999</v>
+        <v>8530.200000000001</v>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>0.19%</t>
+          <t>1.96%</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>03/24</t>
+          <t>03/25</t>
         </is>
       </c>
     </row>
@@ -793,16 +793,16 @@
         </is>
       </c>
       <c r="C15" t="n">
-        <v>72696.39</v>
+        <v>74068.45</v>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>-2.46%</t>
+          <t>1.89%</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>03/23</t>
+          <t>03/24</t>
         </is>
       </c>
     </row>
@@ -818,16 +818,16 @@
         </is>
       </c>
       <c r="C16" t="n">
-        <v>4317.6</v>
+        <v>4568.8</v>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>-5.53%</t>
+          <t>3.74%</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>03/23</t>
+          <t>03/24</t>
         </is>
       </c>
     </row>
@@ -843,16 +843,16 @@
         </is>
       </c>
       <c r="C17" t="n">
-        <v>91.61</v>
+        <v>87.23</v>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>-6.82%</t>
+          <t>-1.02%</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>03/23</t>
+          <t>03/24</t>
         </is>
       </c>
     </row>
@@ -868,16 +868,16 @@
         </is>
       </c>
       <c r="C18" t="n">
-        <v>5.41</v>
+        <v>5.58</v>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>1.21%</t>
+          <t>2.55%</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>03/23</t>
+          <t>03/24</t>
         </is>
       </c>
     </row>
@@ -893,16 +893,16 @@
         </is>
       </c>
       <c r="C19" t="n">
-        <v>66.93000000000001</v>
+        <v>74.37</v>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>-3.51%</t>
+          <t>7.71%</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>03/23</t>
+          <t>03/24</t>
         </is>
       </c>
     </row>
@@ -918,16 +918,16 @@
         </is>
       </c>
       <c r="C20" t="n">
-        <v>1166</v>
+        <v>1154</v>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>0.41%</t>
+          <t>-0.82%</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>03/23</t>
+          <t>03/24</t>
         </is>
       </c>
     </row>
@@ -943,16 +943,16 @@
         </is>
       </c>
       <c r="C21" t="n">
-        <v>463</v>
+        <v>459.25</v>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>-0.54%</t>
+          <t>-0.05%</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>03/23</t>
+          <t>03/24</t>
         </is>
       </c>
     </row>
@@ -968,16 +968,16 @@
         </is>
       </c>
       <c r="C22" t="n">
-        <v>595.25</v>
+        <v>585.75</v>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>0.0%</t>
+          <t>-0.34%</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>03/23</t>
+          <t>03/24</t>
         </is>
       </c>
     </row>
@@ -993,16 +993,16 @@
         </is>
       </c>
       <c r="C23" t="n">
-        <v>4.33</v>
+        <v>4.39</v>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>-5.7bp</t>
+          <t>5.8bp</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>03/23</t>
+          <t>03/24</t>
         </is>
       </c>
     </row>
@@ -1018,16 +1018,16 @@
         </is>
       </c>
       <c r="C24" t="n">
-        <v>70524.8</v>
+        <v>70789.73</v>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>3.95%</t>
+          <t>-0.18%</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>03/24</t>
+          <t>03/25</t>
         </is>
       </c>
     </row>
@@ -1043,16 +1043,16 @@
         </is>
       </c>
       <c r="C25" t="n">
-        <v>32.07</v>
+        <v>31.88</v>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>0.16%</t>
+          <t>0.06%</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>03/24</t>
+          <t>03/25</t>
         </is>
       </c>
     </row>
@@ -1072,12 +1072,12 @@
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>-0.54%</t>
+          <t>-0.08%</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>03/24</t>
+          <t>03/25</t>
         </is>
       </c>
     </row>
@@ -1097,12 +1097,12 @@
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>0.24%</t>
+          <t>0.2%</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>03/24</t>
+          <t>03/25</t>
         </is>
       </c>
     </row>
@@ -1118,16 +1118,16 @@
         </is>
       </c>
       <c r="C28" t="n">
-        <v>158.61</v>
+        <v>158.62</v>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>-0.39%</t>
+          <t>0.09%</t>
         </is>
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>03/24</t>
+          <t>03/25</t>
         </is>
       </c>
     </row>
@@ -1143,16 +1143,16 @@
         </is>
       </c>
       <c r="C29" t="n">
-        <v>99.37</v>
+        <v>99.08</v>
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>-0.28%</t>
+          <t>0.13%</t>
         </is>
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>03/23</t>
+          <t>03/24</t>
         </is>
       </c>
     </row>

</xml_diff>